<commit_message>
Editacia exportu do excelu
</commit_message>
<xml_diff>
--- a/RozvrhUniza/RozvrhDverePriklad.xlsx
+++ b/RozvrhUniza/RozvrhDverePriklad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sources\Repos\RozvrhUniza\RozvrhUniza\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34CF4600-5D5E-4279-911B-26FF450EB8D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5081821-B8C2-4781-96E8-2422802DDC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="zdroj" sheetId="1" r:id="rId1"/>
@@ -715,62 +715,62 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1086,222 +1086,222 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BE30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" customWidth="1"/>
-    <col min="2" max="5" width="1.28515625" hidden="1" customWidth="1"/>
-    <col min="6" max="57" width="1.140625" customWidth="1"/>
+    <col min="1" max="1" width="7.5546875" customWidth="1"/>
+    <col min="2" max="5" width="1.33203125" hidden="1" customWidth="1"/>
+    <col min="6" max="57" width="1.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="53" t="s">
+    <row r="1" spans="1:57" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="54"/>
-      <c r="O1" s="54"/>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="54"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="54"/>
-      <c r="X1" s="54"/>
-      <c r="Y1" s="54"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
-      <c r="AB1" s="54"/>
-      <c r="AC1" s="54"/>
-      <c r="AD1" s="54"/>
-      <c r="AE1" s="54"/>
-      <c r="AF1" s="54"/>
-      <c r="AG1" s="54"/>
-      <c r="AH1" s="54"/>
-      <c r="AI1" s="54"/>
-      <c r="AJ1" s="54"/>
-      <c r="AK1" s="54"/>
-      <c r="AL1" s="54"/>
-      <c r="AM1" s="54"/>
-      <c r="AN1" s="54"/>
-      <c r="AO1" s="54"/>
-      <c r="AP1" s="54"/>
-      <c r="AQ1" s="54"/>
-      <c r="AR1" s="54"/>
-      <c r="AS1" s="54"/>
-      <c r="AT1" s="54"/>
-      <c r="AU1" s="54"/>
-      <c r="AV1" s="54"/>
-      <c r="AW1" s="54"/>
-      <c r="AX1" s="54"/>
-      <c r="AY1" s="54"/>
-      <c r="AZ1" s="54"/>
-      <c r="BA1" s="54"/>
-      <c r="BB1" s="54"/>
-      <c r="BC1" s="54"/>
-      <c r="BD1" s="54"/>
-      <c r="BE1" s="54"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
+      <c r="AK1" s="44"/>
+      <c r="AL1" s="44"/>
+      <c r="AM1" s="44"/>
+      <c r="AN1" s="44"/>
+      <c r="AO1" s="44"/>
+      <c r="AP1" s="44"/>
+      <c r="AQ1" s="44"/>
+      <c r="AR1" s="44"/>
+      <c r="AS1" s="44"/>
+      <c r="AT1" s="44"/>
+      <c r="AU1" s="44"/>
+      <c r="AV1" s="44"/>
+      <c r="AW1" s="44"/>
+      <c r="AX1" s="44"/>
+      <c r="AY1" s="44"/>
+      <c r="AZ1" s="44"/>
+      <c r="BA1" s="44"/>
+      <c r="BB1" s="44"/>
+      <c r="BC1" s="44"/>
+      <c r="BD1" s="44"/>
+      <c r="BE1" s="44"/>
     </row>
-    <row r="2" spans="1:57" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
-      <c r="Q2" s="54"/>
-      <c r="R2" s="54"/>
-      <c r="S2" s="54"/>
-      <c r="T2" s="54"/>
-      <c r="U2" s="54"/>
-      <c r="V2" s="54"/>
-      <c r="W2" s="54"/>
-      <c r="X2" s="54"/>
-      <c r="Y2" s="54"/>
-      <c r="Z2" s="54"/>
-      <c r="AA2" s="54"/>
-      <c r="AB2" s="54"/>
-      <c r="AC2" s="54"/>
-      <c r="AD2" s="54"/>
-      <c r="AE2" s="54"/>
-      <c r="AF2" s="54"/>
-      <c r="AG2" s="54"/>
-      <c r="AH2" s="54"/>
-      <c r="AI2" s="54"/>
-      <c r="AJ2" s="54"/>
-      <c r="AK2" s="54"/>
-      <c r="AL2" s="54"/>
-      <c r="AM2" s="54"/>
-      <c r="AN2" s="54"/>
-      <c r="AO2" s="54"/>
-      <c r="AP2" s="54"/>
-      <c r="AQ2" s="54"/>
-      <c r="AR2" s="54"/>
-      <c r="AS2" s="54"/>
-      <c r="AT2" s="54"/>
-      <c r="AU2" s="54"/>
-      <c r="AV2" s="54"/>
-      <c r="AW2" s="54"/>
-      <c r="AX2" s="54"/>
-      <c r="AY2" s="54"/>
-      <c r="AZ2" s="54"/>
-      <c r="BA2" s="54"/>
-      <c r="BB2" s="54"/>
-      <c r="BC2" s="54"/>
-      <c r="BD2" s="54"/>
-      <c r="BE2" s="54"/>
+    <row r="2" spans="1:57" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="43"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
+      <c r="S2" s="44"/>
+      <c r="T2" s="44"/>
+      <c r="U2" s="44"/>
+      <c r="V2" s="44"/>
+      <c r="W2" s="44"/>
+      <c r="X2" s="44"/>
+      <c r="Y2" s="44"/>
+      <c r="Z2" s="44"/>
+      <c r="AA2" s="44"/>
+      <c r="AB2" s="44"/>
+      <c r="AC2" s="44"/>
+      <c r="AD2" s="44"/>
+      <c r="AE2" s="44"/>
+      <c r="AF2" s="44"/>
+      <c r="AG2" s="44"/>
+      <c r="AH2" s="44"/>
+      <c r="AI2" s="44"/>
+      <c r="AJ2" s="44"/>
+      <c r="AK2" s="44"/>
+      <c r="AL2" s="44"/>
+      <c r="AM2" s="44"/>
+      <c r="AN2" s="44"/>
+      <c r="AO2" s="44"/>
+      <c r="AP2" s="44"/>
+      <c r="AQ2" s="44"/>
+      <c r="AR2" s="44"/>
+      <c r="AS2" s="44"/>
+      <c r="AT2" s="44"/>
+      <c r="AU2" s="44"/>
+      <c r="AV2" s="44"/>
+      <c r="AW2" s="44"/>
+      <c r="AX2" s="44"/>
+      <c r="AY2" s="44"/>
+      <c r="AZ2" s="44"/>
+      <c r="BA2" s="44"/>
+      <c r="BB2" s="44"/>
+      <c r="BC2" s="44"/>
+      <c r="BD2" s="44"/>
+      <c r="BE2" s="44"/>
     </row>
-    <row r="3" spans="1:57" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:57" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="45" t="s">
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="45" t="s">
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="45" t="s">
+      <c r="K3" s="52"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="45" t="s">
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="55"/>
+      <c r="R3" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="S3" s="46"/>
-      <c r="T3" s="46"/>
-      <c r="U3" s="47"/>
-      <c r="V3" s="45" t="s">
+      <c r="S3" s="52"/>
+      <c r="T3" s="52"/>
+      <c r="U3" s="53"/>
+      <c r="V3" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="W3" s="46"/>
-      <c r="X3" s="46"/>
-      <c r="Y3" s="47"/>
-      <c r="Z3" s="45" t="s">
+      <c r="W3" s="52"/>
+      <c r="X3" s="52"/>
+      <c r="Y3" s="53"/>
+      <c r="Z3" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="AA3" s="46"/>
-      <c r="AB3" s="46"/>
-      <c r="AC3" s="47"/>
-      <c r="AD3" s="45" t="s">
+      <c r="AA3" s="52"/>
+      <c r="AB3" s="52"/>
+      <c r="AC3" s="53"/>
+      <c r="AD3" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="AE3" s="46"/>
-      <c r="AF3" s="46"/>
-      <c r="AG3" s="47"/>
-      <c r="AH3" s="45" t="s">
+      <c r="AE3" s="52"/>
+      <c r="AF3" s="52"/>
+      <c r="AG3" s="53"/>
+      <c r="AH3" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="AI3" s="46"/>
-      <c r="AJ3" s="46"/>
-      <c r="AK3" s="47"/>
-      <c r="AL3" s="45" t="s">
+      <c r="AI3" s="52"/>
+      <c r="AJ3" s="52"/>
+      <c r="AK3" s="53"/>
+      <c r="AL3" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="AM3" s="46"/>
-      <c r="AN3" s="46"/>
-      <c r="AO3" s="47"/>
-      <c r="AP3" s="45" t="s">
+      <c r="AM3" s="52"/>
+      <c r="AN3" s="52"/>
+      <c r="AO3" s="53"/>
+      <c r="AP3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="AQ3" s="46"/>
-      <c r="AR3" s="46"/>
-      <c r="AS3" s="47"/>
-      <c r="AT3" s="48" t="s">
+      <c r="AQ3" s="52"/>
+      <c r="AR3" s="52"/>
+      <c r="AS3" s="53"/>
+      <c r="AT3" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="AU3" s="49"/>
-      <c r="AV3" s="49"/>
-      <c r="AW3" s="50"/>
-      <c r="AX3" s="48" t="s">
+      <c r="AU3" s="57"/>
+      <c r="AV3" s="57"/>
+      <c r="AW3" s="58"/>
+      <c r="AX3" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="AY3" s="49"/>
-      <c r="AZ3" s="49"/>
-      <c r="BA3" s="50"/>
-      <c r="BB3" s="48" t="s">
+      <c r="AY3" s="57"/>
+      <c r="AZ3" s="57"/>
+      <c r="BA3" s="58"/>
+      <c r="BB3" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="BC3" s="49"/>
-      <c r="BD3" s="49"/>
-      <c r="BE3" s="50"/>
+      <c r="BC3" s="57"/>
+      <c r="BD3" s="57"/>
+      <c r="BE3" s="58"/>
     </row>
-    <row r="4" spans="1:57" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="55" t="s">
+    <row r="4" spans="1:57" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="45" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="8"/>
@@ -1361,8 +1361,8 @@
       <c r="BD4" s="21"/>
       <c r="BE4" s="22"/>
     </row>
-    <row r="5" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="56"/>
+    <row r="5" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="46"/>
       <c r="B5" s="6"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -1420,8 +1420,8 @@
       <c r="BD5" s="23"/>
       <c r="BE5" s="24"/>
     </row>
-    <row r="6" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
+    <row r="6" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="47" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="6"/>
@@ -1481,8 +1481,8 @@
       <c r="BD6" s="21"/>
       <c r="BE6" s="22"/>
     </row>
-    <row r="7" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56"/>
+    <row r="7" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="46"/>
       <c r="B7" s="6"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -1540,11 +1540,11 @@
       <c r="BD7" s="23"/>
       <c r="BE7" s="24"/>
     </row>
-    <row r="8" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+    <row r="8" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="51"/>
+      <c r="B8" s="59"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="17"/>
@@ -1601,9 +1601,9 @@
       <c r="BD8" s="21"/>
       <c r="BE8" s="22"/>
     </row>
-    <row r="9" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="44"/>
-      <c r="B9" s="52"/>
+    <row r="9" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="61"/>
+      <c r="B9" s="60"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="19"/>
@@ -1660,8 +1660,8 @@
       <c r="BD9" s="23"/>
       <c r="BE9" s="24"/>
     </row>
-    <row r="10" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="43" t="s">
+    <row r="10" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="47" t="s">
         <v>1</v>
       </c>
       <c r="B10" s="5"/>
@@ -1721,8 +1721,8 @@
       <c r="BD10" s="21"/>
       <c r="BE10" s="22"/>
     </row>
-    <row r="11" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="44"/>
+    <row r="11" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="61"/>
       <c r="B11" s="5"/>
       <c r="C11" s="4"/>
       <c r="D11" s="9"/>
@@ -1780,8 +1780,8 @@
       <c r="BD11" s="23"/>
       <c r="BE11" s="24"/>
     </row>
-    <row r="12" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+    <row r="12" spans="1:57" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B12" s="5"/>
@@ -1841,8 +1841,8 @@
       <c r="BD12" s="21"/>
       <c r="BE12" s="22"/>
     </row>
-    <row r="13" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="44"/>
+    <row r="13" spans="1:57" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="61"/>
       <c r="B13" s="11"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -1900,9 +1900,9 @@
       <c r="BD13" s="23"/>
       <c r="BE13" s="24"/>
     </row>
-    <row r="14" spans="1:57" s="1" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:57" s="1" customFormat="1" ht="12" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="42"/>
       <c r="B16" s="42"/>
       <c r="C16" s="42"/>
@@ -1961,7 +1961,7 @@
       <c r="BD16" s="42"/>
       <c r="BE16" s="42"/>
     </row>
-    <row r="17" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="42"/>
       <c r="B17" s="42"/>
       <c r="C17" s="42"/>
@@ -2020,7 +2020,7 @@
       <c r="BD17" s="42"/>
       <c r="BE17" s="42"/>
     </row>
-    <row r="18" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="27"/>
       <c r="B18" s="37"/>
       <c r="C18" s="37"/>
@@ -2079,7 +2079,7 @@
       <c r="BD18" s="26"/>
       <c r="BE18" s="26"/>
     </row>
-    <row r="19" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="39"/>
       <c r="B19" s="28"/>
       <c r="C19" s="28"/>
@@ -2138,7 +2138,7 @@
       <c r="BD19" s="29"/>
       <c r="BE19" s="29"/>
     </row>
-    <row r="20" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="41"/>
       <c r="B20" s="28"/>
       <c r="C20" s="28"/>
@@ -2197,7 +2197,7 @@
       <c r="BD20" s="29"/>
       <c r="BE20" s="29"/>
     </row>
-    <row r="21" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="39"/>
       <c r="B21" s="28"/>
       <c r="C21" s="28"/>
@@ -2256,7 +2256,7 @@
       <c r="BD21" s="29"/>
       <c r="BE21" s="29"/>
     </row>
-    <row r="22" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="41"/>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -2315,7 +2315,7 @@
       <c r="BD22" s="29"/>
       <c r="BE22" s="29"/>
     </row>
-    <row r="23" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="39"/>
       <c r="B23" s="40"/>
       <c r="C23" s="28"/>
@@ -2374,7 +2374,7 @@
       <c r="BD23" s="29"/>
       <c r="BE23" s="29"/>
     </row>
-    <row r="24" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="39"/>
       <c r="B24" s="40"/>
       <c r="C24" s="31"/>
@@ -2433,7 +2433,7 @@
       <c r="BD24" s="29"/>
       <c r="BE24" s="29"/>
     </row>
-    <row r="25" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39"/>
       <c r="B25" s="32"/>
       <c r="C25" s="32"/>
@@ -2492,7 +2492,7 @@
       <c r="BD25" s="29"/>
       <c r="BE25" s="29"/>
     </row>
-    <row r="26" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="39"/>
       <c r="B26" s="32"/>
       <c r="C26" s="32"/>
@@ -2551,7 +2551,7 @@
       <c r="BD26" s="29"/>
       <c r="BE26" s="29"/>
     </row>
-    <row r="27" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="39"/>
       <c r="B27" s="32"/>
       <c r="C27" s="32"/>
@@ -2610,7 +2610,7 @@
       <c r="BD27" s="29"/>
       <c r="BE27" s="29"/>
     </row>
-    <row r="28" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="39"/>
       <c r="B28" s="28"/>
       <c r="C28" s="33"/>
@@ -2669,10 +2669,15 @@
       <c r="BD28" s="29"/>
       <c r="BE28" s="29"/>
     </row>
-    <row r="29" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="BB3:BE3"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A8:A9"/>
     <mergeCell ref="A1:BE2"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="A6:A7"/>
@@ -2689,11 +2694,6 @@
     <mergeCell ref="Z3:AC3"/>
     <mergeCell ref="AD3:AG3"/>
     <mergeCell ref="AX3:BA3"/>
-    <mergeCell ref="BB3:BE3"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A8:A9"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" r:id="rId1"/>

</xml_diff>